<commit_message>
chore(output): update audit rubric spreadsheet
</commit_message>
<xml_diff>
--- a/output/audit_rubric.xlsx
+++ b/output/audit_rubric.xlsx
@@ -35,7 +35,7 @@
     <t>All models</t>
   </si>
   <si>
-    <t>No model produced expected revenue of $439,918.30; all computed from slip inventory ($342,358.85) or used July actual ($319,760.05) without accounting for underbilled amounts.</t>
+    <t>No model produced expected revenue of $439,918.30.</t>
   </si>
   <si>
     <t>R-02</t>
@@ -53,7 +53,7 @@
     <t>Rsponse 1</t>
   </si>
   <si>
-    <t>Rsponse 1 calculated $360,817.12 using total_amount (inclusive of tax) instead of amount field ($319,760.05); also used incorrect filename.</t>
+    <t>Rsponse 1 calculated $360,817.12 using total_amount instead of amount field.</t>
   </si>
   <si>
     <t>R-03</t>
@@ -71,7 +71,7 @@
     <t>CE-03: Monthly Exposure</t>
   </si>
   <si>
-    <t>No model computed exposure as $439,918.30 minus $319,760.05; most reported no exposure or used incorrect arithmetic.</t>
+    <t>No model computed exposure as $439,918.30 minus $319,760.05.</t>
   </si>
   <si>
     <t>R-04</t>
@@ -89,7 +89,7 @@
     <t>CE-04: Annualized Exposure</t>
   </si>
   <si>
-    <t>No model computed annualized exposure as $120,158.25 multiplied by 12 months.</t>
+    <t>No model computed annualized exposure as $120,158.25 x 12.</t>
   </si>
   <si>
     <t>R-05</t>
@@ -107,7 +107,7 @@
     <t>CE-05: Missing Export Slips</t>
   </si>
   <si>
-    <t>All models failed to identify 317-slip coverage gap and $99,629.80 baseline; conflated with revenue leakage without verifying term/prepayment.</t>
+    <t>All models failed to identify 317-slip coverage gap.</t>
   </si>
   <si>
     <t>R-06</t>
@@ -116,7 +116,7 @@
     <t>Baseline Floor Methodology</t>
   </si>
   <si>
-    <t>Model explicitly states 317 missing slips represent unverified coverage, not booked leakage, requiring term/prepayment evidence</t>
+    <t>Model explicitly states 317 missing slips represent unverified coverage not booked leakage</t>
   </si>
   <si>
     <t>70</t>
@@ -125,7 +125,7 @@
     <t>CE-06: Baseline Floor</t>
   </si>
   <si>
-    <t>All models incorrectly treated 317 missing slips as automatic leakage; requires evidence of term or prepayment before classifying as leakage.</t>
+    <t>All models treated 317 missing slips as automatic leakage.</t>
   </si>
   <si>
     <t>R-07</t>
@@ -137,13 +137,13 @@
     <t>Skip-Proof Failures</t>
   </si>
   <si>
-    <t>Model identifies exactly 19 skip events with documentation_attached=N in audit window</t>
+    <t>Model identifies exactly 19 skip events with documentation_attached=N</t>
   </si>
   <si>
     <t>CE-07: Skip-Proof Failures</t>
   </si>
   <si>
-    <t>All models failed to identify exactly 19 skip events lacking same-day proof; reported different counts or did not apply SO 15-3 s.3.2 correctly.</t>
+    <t>All models failed to identify exactly 19 skip events.</t>
   </si>
   <si>
     <t>R-08</t>
@@ -152,13 +152,13 @@
     <t>Unsupported LOA Entries</t>
   </si>
   <si>
-    <t>Model identifies 11 LOA amendments post-Aug 2022 with no source document and no downstream skip use</t>
+    <t>Model identifies 11 LOA amendments post-Aug 2022 with no source document</t>
   </si>
   <si>
     <t>CE-08: Unsupported LOA</t>
   </si>
   <si>
-    <t>All models failed to identify exactly 11 unsupported LOA entries; either included supported amendments or missed unsupported ones.</t>
+    <t>All models failed to identify exactly 11 unsupported LOA entries.</t>
   </si>
   <si>
     <t>R-09</t>
@@ -167,13 +167,13 @@
     <t>Unresolved Cases</t>
   </si>
   <si>
-    <t>Model identifies WL-01999 and WL-02085 as unresolved with justification</t>
+    <t>Model identifies WL-01999 and WL-02085 as unresolved</t>
   </si>
   <si>
     <t>CE-09: Unresolved Cases</t>
   </si>
   <si>
-    <t>All models failed to identify WL-01999 and WL-02085 as unresolved; these have unsupported LOAs with zero skip events and stale/zero offers.</t>
+    <t>All models failed to identify WL-01999 and WL-02085 as unresolved.</t>
   </si>
   <si>
     <t>R-10</t>
@@ -182,13 +182,13 @@
     <t>Triage Distribution</t>
   </si>
   <si>
-    <t>Model reports 7 Priority 1, 16 Priority 2, 9 Priority 3 exceptions (32 total)</t>
+    <t>Model reports 7 Priority 1, 16 Priority 2, 9 Priority 3 (32 total)</t>
   </si>
   <si>
     <t>CE-10: Triage Distribution</t>
   </si>
   <si>
-    <t>No model produced correct triage distribution of 7P1/16P2/9P3; most collapsed all exceptions into one tier or used incorrect logic.</t>
+    <t>No model produced correct triage distribution.</t>
   </si>
   <si>
     <t>R-11</t>
@@ -203,46 +203,46 @@
     <t>CE-11: Priority Accounts</t>
   </si>
   <si>
-    <t>No model correctly identified all 7 Priority 1 accounts; missed WL-02319 (late support), WL-02712 (invalid code), WL-01999, or WL-02085.</t>
+    <t>No model correctly identified all 7 Priority 1 accounts.</t>
   </si>
   <si>
     <t>R-12</t>
   </si>
   <si>
-    <t>Legal Basis for Skip Decisions</t>
-  </si>
-  <si>
-    <t>Model cites Standing Order 15-3 s.3.2-3.5 and Appeal 2018-3 as governing legal framework</t>
+    <t>Legal Basis</t>
+  </si>
+  <si>
+    <t>Model cites SO 15-3 s.3.2-3.5 and Appeal 2018-3 as governing framework</t>
   </si>
   <si>
     <t>CE-15: Legal Basis</t>
   </si>
   <si>
-    <t>All models failed to cite both SO 15-3 and Appeal 2018-3; most referenced only one or neither; none explained burden-of-proof transfer.</t>
+    <t>All models failed to cite both authorities.</t>
   </si>
   <si>
     <t>R-13</t>
   </si>
   <si>
-    <t>File/Identity Mismatch Detection</t>
-  </si>
-  <si>
-    <t>Model identifies WL-02877 and WL-03102 as file/event identity mismatches</t>
+    <t>Identity Mismatch</t>
+  </si>
+  <si>
+    <t>Model identifies WL-02877 and WL-03102 as file/event mismatches</t>
   </si>
   <si>
     <t>CE-13: Identity Mismatch</t>
   </si>
   <si>
-    <t>All models failed to detect WL-02877 supports EW-0702 (not GW-1012) and WL-03102 supports EW-0620 (not LP-0806); LOA support was valid.</t>
+    <t>All models failed to detect identity mismatches.</t>
   </si>
   <si>
     <t>R-14</t>
   </si>
   <si>
-    <t>Late Support Detection</t>
-  </si>
-  <si>
-    <t>Model identifies WL-02319 as having supporting record dated after slip was worked</t>
+    <t>Late Support</t>
+  </si>
+  <si>
+    <t>Model identifies WL-02319 late supporting record</t>
   </si>
   <si>
     <t>65</t>
@@ -251,7 +251,7 @@
     <t>CE-14: Late Support</t>
   </si>
   <si>
-    <t>All models failed to identify WL-02319 where supporting record was dated 3 days after slip worked; per-occurrence violation of SO 15-3 s.3.3.</t>
+    <t>All models failed to identify WL-02319.</t>
   </si>
   <si>
     <t>R-15</t>
@@ -260,52 +260,52 @@
     <t>Billing Reconciliation</t>
   </si>
   <si>
-    <t>Rate Class Identification</t>
-  </si>
-  <si>
-    <t>Model applies $10.40/ft-mo for covered basins and $7.55/ft-mo for open basins per Resolution 2022-06</t>
+    <t>Rate Class</t>
+  </si>
+  <si>
+    <t>Model applies $10.40 covered / $7.55 open per Res 2022-06</t>
   </si>
   <si>
     <t>CE-14: Billing Rates</t>
   </si>
   <si>
-    <t>No model correctly identified/applied post-adoption rates of $10.40/$7.55; Rsponse 1 used pre-adoption rates ($9.85/$7.10) and misidentified effective date.</t>
+    <t>No model correctly applied post-adoption rates.</t>
   </si>
   <si>
     <t>R-16</t>
   </si>
   <si>
-    <t>Billable Length Formula</t>
-  </si>
-  <si>
-    <t>Model applies MAX(rounded-up check-in LOA, posted slip length) for July 2026 billing</t>
-  </si>
-  <si>
-    <t>All models failed to apply MAX(rounded-up LOA, posted slip length); most used raw slip size or raw LOA without MAX rule.</t>
+    <t>Billable Length</t>
+  </si>
+  <si>
+    <t>Model applies MAX(rounded-up LOA, posted slip length)</t>
+  </si>
+  <si>
+    <t>All models failed to apply MAX formula.</t>
   </si>
   <si>
     <t>R-17</t>
   </si>
   <si>
-    <t>Pre/Post Adoption Rate Transition</t>
-  </si>
-  <si>
-    <t>Model correctly identifies August 1, 2022 as adoption date and applies post-adoption rates to July 2026</t>
-  </si>
-  <si>
-    <t>All models failed to anchor rate transition to August 1, 2022; some used pre-adoption rates for July 2026.</t>
+    <t>Rate Transition</t>
+  </si>
+  <si>
+    <t>Model identifies Aug 1, 2022 as adoption date</t>
+  </si>
+  <si>
+    <t>All models failed to anchor rate transition date.</t>
   </si>
   <si>
     <t>R-18</t>
   </si>
   <si>
-    <t>Coverage by Basin Analysis</t>
-  </si>
-  <si>
-    <t>Model reports occupied count vs July rows vs unscored per basin for all 5 basins</t>
-  </si>
-  <si>
-    <t>All models failed to produce basin-level coverage analysis showing occupied, July-tested, and unscored counts per basin.</t>
+    <t>Basin Coverage</t>
+  </si>
+  <si>
+    <t>Model reports occupied vs July rows vs unscored per basin</t>
+  </si>
+  <si>
+    <t>All models failed basin-level coverage analysis.</t>
   </si>
   <si>
     <t>R-19</t>
@@ -314,28 +314,28 @@
     <t>Aging Analysis</t>
   </si>
   <si>
-    <t>Over-90-Day Account Count</t>
-  </si>
-  <si>
-    <t>Model identifies exactly 6 active holders over 90 days past due</t>
+    <t>Over-90 Count</t>
+  </si>
+  <si>
+    <t>Model identifies exactly 6 holders over 90 days</t>
   </si>
   <si>
     <t>CE-11: Aging &gt;90</t>
   </si>
   <si>
-    <t>All models failed to identify exactly 6 overdue accounts; most reported different counts or used incorrect date thresholds.</t>
+    <t>All models failed to identify exactly 6 overdue accounts.</t>
   </si>
   <si>
     <t>R-20</t>
   </si>
   <si>
-    <t>Over-90-Day Balance</t>
-  </si>
-  <si>
-    <t>Model reports $4,368.00 as total balance for 6 overdue accounts</t>
-  </si>
-  <si>
-    <t>All models failed to compute correct over-90 balance of $4,368.00; summed incorrectly or included non-overdue amounts.</t>
+    <t>Over-90 Balance</t>
+  </si>
+  <si>
+    <t>Model reports $4,368.00 as total balance</t>
+  </si>
+  <si>
+    <t>All models failed to compute correct balance.</t>
   </si>
   <si>
     <t>R-21</t>
@@ -344,25 +344,25 @@
     <t>Missing from Aging</t>
   </si>
   <si>
-    <t>Model identifies 826 occupied accounts absent from AR aging report (out of 1,086)</t>
+    <t>Model identifies 826 occupied accounts absent from aging</t>
   </si>
   <si>
     <t>CE-12: Missing from Aging</t>
   </si>
   <si>
-    <t>All models failed to identify 826 missing accounts from aging; 260 in aging is correct but 826 gap universally missed.</t>
+    <t>All models failed to identify 826 missing accounts.</t>
   </si>
   <si>
     <t>R-22</t>
   </si>
   <si>
-    <t>Aging Bucket Reconciliation</t>
-  </si>
-  <si>
-    <t>Model reconciles 91-120 day bucket ($2,932.80) and 120+ bucket ($1,435.20) to over-90 total ($4,368.00)</t>
-  </si>
-  <si>
-    <t>All models failed to verify 91-120 ($2,932.80) plus 120+ ($1,435.20) sums to $4,368.00.</t>
+    <t>Aging Reconciliation</t>
+  </si>
+  <si>
+    <t>Model reconciles 91-120 ($2,932.80) + 120+ ($1,435.20) = $4,368.00</t>
+  </si>
+  <si>
+    <t>All models failed aging bucket reconciliation.</t>
   </si>
   <si>
     <t>R-23</t>
@@ -371,40 +371,40 @@
     <t>Subledger Reconciliation</t>
   </si>
   <si>
-    <t>Subledger Error Count</t>
-  </si>
-  <si>
-    <t>Model identifies 39 arithmetic discrepancies in subledger billing records</t>
+    <t>Error Count</t>
+  </si>
+  <si>
+    <t>Model identifies 39 subledger discrepancies</t>
   </si>
   <si>
     <t>CE-13: Subledger Errors</t>
   </si>
   <si>
-    <t>All models failed to identify 39 subledger math errors against verified bucket total.</t>
+    <t>All models failed to identify 39 errors.</t>
   </si>
   <si>
     <t>R-24</t>
   </si>
   <si>
-    <t>Control Gap Calculation</t>
-  </si>
-  <si>
-    <t>Model reports $17,108.00 as control gap between subledger errors and true total</t>
-  </si>
-  <si>
-    <t>All models failed to calculate control gap of $17,108.00 (difference between $147,836.00 true total and error-impacted amount).</t>
+    <t>Control Gap</t>
+  </si>
+  <si>
+    <t>Model reports $17,108.00 control gap</t>
+  </si>
+  <si>
+    <t>All models failed to calculate control gap.</t>
   </si>
   <si>
     <t>R-25</t>
   </si>
   <si>
-    <t>True Bucket Total</t>
-  </si>
-  <si>
-    <t>Model reports $147,836.00 as verified subledger total before errors</t>
-  </si>
-  <si>
-    <t>All models failed to establish true bucket total of $147,836.00 as benchmark for measuring subledger errors.</t>
+    <t>True Total</t>
+  </si>
+  <si>
+    <t>Model reports $147,836.00 verified total</t>
+  </si>
+  <si>
+    <t>All models failed to establish true total.</t>
   </si>
   <si>
     <t>R-26</t>
@@ -416,7 +416,7 @@
     <t>Zero-Width Characters</t>
   </si>
   <si>
-    <t>Deliverable contains no U+2060 or other invisible characters in filenames or body text</t>
+    <t>No U+2060 in deliverables</t>
   </si>
   <si>
     <t>-100</t>
@@ -428,7 +428,7 @@
     <t>Prompt Integrity</t>
   </si>
   <si>
-    <t>Original prompt contained 17 U+2060 zero-width characters surrounding every filename; invisible but breaks file matching.</t>
+    <t>Original prompt had 17 zero-width characters.</t>
   </si>
   <si>
     <t>R-27</t>
@@ -437,22 +437,22 @@
     <t>Filename Accuracy</t>
   </si>
   <si>
-    <t>All filenames in Required Files list match actual workspace filenames exactly (case, separators, spelling)</t>
-  </si>
-  <si>
-    <t>Original prompt had 14 filenames with wrong case, typo in WL-03390_Skip-justificaton.pdf (missing i), and separator inconsistencies.</t>
+    <t>All filenames match workspace exactly</t>
+  </si>
+  <si>
+    <t>Original had wrong case, typos, separators.</t>
   </si>
   <si>
     <t>R-28</t>
   </si>
   <si>
-    <t>Required Files Completeness</t>
-  </si>
-  <si>
-    <t>Required Files list includes billing_transactions_2022_2026.csv and appeal_2018-3_decision.pdf</t>
-  </si>
-  <si>
-    <t>Original Required Files list omitted billing_transactions_2022_2026.csv (46,800 rows, primary billing data) and appeal_2018-3_decision.pdf (legal precedent).</t>
+    <t>Required Files</t>
+  </si>
+  <si>
+    <t>List includes billing_transactions_2022_2026.csv and appeal_2018-3_decision.pdf</t>
+  </si>
+  <si>
+    <t>Omitted two required files.</t>
   </si>
   <si>
     <t>R-29</t>
@@ -461,28 +461,28 @@
     <t>Deliverable Completeness</t>
   </si>
   <si>
-    <t>Memo description is complete and not truncated; covers all specified deliverable requirements</t>
+    <t>Memo not truncated; covers all requirements</t>
   </si>
   <si>
     <t>-80</t>
   </si>
   <si>
-    <t>Original memo description was truncated without specifying what to summarize or deliver format; later addition may be insufficient.</t>
+    <t>Memo description was truncated.</t>
   </si>
   <si>
     <t>R-30</t>
   </si>
   <si>
-    <t>Undefined Terms Explained</t>
-  </si>
-  <si>
-    <t>All domain-specific terms (check-in measurements, contemporaneous proof of eligibility, etc.) are defined or sourced</t>
+    <t>Undefined Terms</t>
+  </si>
+  <si>
+    <t>Domain terms defined or sourced</t>
   </si>
   <si>
     <t>-70</t>
   </si>
   <si>
-    <t>Original prompt used undefined terms including check-in measurements and contemporaneous proof of eligibility.</t>
+    <t>Undefined terms used.</t>
   </si>
   <si>
     <t>R-31</t>
@@ -491,10 +491,10 @@
     <t>Constraints</t>
   </si>
   <si>
-    <t>Negative Constraints Present</t>
-  </si>
-  <si>
-    <t>Prompt includes must-not constraints (data is not to be excluded, assumptions are not to be made, etc.)</t>
+    <t>Negative Constraints</t>
+  </si>
+  <si>
+    <t>Prompt includes must-not rules</t>
   </si>
   <si>
     <t>60</t>
@@ -503,52 +503,52 @@
     <t>CE-06: Constraints</t>
   </si>
   <si>
-    <t>Original prompt had no negative constraints which Buckeye requires; models had no guardrails against assumptions.</t>
+    <t>No negative constraints in original.</t>
   </si>
   <si>
     <t>R-32</t>
   </si>
   <si>
-    <t>Relative Date Anchored</t>
-  </si>
-  <si>
-    <t>All date-relative terms anchored to August 1, 2026 as audit date</t>
+    <t>Date Anchored</t>
+  </si>
+  <si>
+    <t>Terms anchored to Aug 1, 2026</t>
   </si>
   <si>
     <t>CE-05: Constraints</t>
   </si>
   <si>
-    <t>Original prompt used 'more than 90 days delinquent' without anchoring to August 1, 2026; models applied inconsistent thresholds.</t>
+    <t>Relative dates not anchored.</t>
   </si>
   <si>
     <t>R-33</t>
   </si>
   <si>
-    <t>Task for amendment_log</t>
-  </si>
-  <si>
-    <t>Prompt provides explicit instruction for amendment_log_2022_2026.csv usage</t>
+    <t>Amendment Log Task</t>
+  </si>
+  <si>
+    <t>Instruction for amendment_log_2022_2026.csv</t>
   </si>
   <si>
     <t>55</t>
   </si>
   <si>
-    <t>Original prompt listed amendment_log but gave no instruction; load-bearing for LOA verification.</t>
+    <t>No task assigned.</t>
   </si>
   <si>
     <t>R-34</t>
   </si>
   <si>
-    <t>Grammar and Terminology</t>
-  </si>
-  <si>
-    <t>Prompt uses correct grammar and consistent terminology (skip vs bypass, applicant possessive, etc.)</t>
+    <t>Grammar</t>
+  </si>
+  <si>
+    <t>Correct grammar and terminology</t>
   </si>
   <si>
     <t>-50</t>
   </si>
   <si>
-    <t>Original prompt had grammar errors including 'Audit all applicants skips' and 'bypass' (data uses 'skip' exclusively).</t>
+    <t>Grammar errors present.</t>
   </si>
   <si>
     <t>Model</t>
@@ -1755,10 +1755,10 @@
         <v>182</v>
       </c>
       <c r="I2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K2" t="s">
         <v>181</v>
@@ -1767,10 +1767,10 @@
         <v>181</v>
       </c>
       <c r="M2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O2" t="s">
         <v>181</v>
@@ -1779,22 +1779,22 @@
         <v>182</v>
       </c>
       <c r="Q2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R2" t="s">
         <v>182</v>
       </c>
       <c r="S2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="T2" t="s">
         <v>181</v>
       </c>
       <c r="U2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="V2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="W2" t="s">
         <v>181</v>
@@ -1806,16 +1806,16 @@
         <v>181</v>
       </c>
       <c r="Z2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AA2" t="s">
         <v>181</v>
       </c>
       <c r="AB2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AD2" t="s">
         <v>181</v>
@@ -1824,7 +1824,7 @@
         <v>181</v>
       </c>
       <c r="AF2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AG2" t="s">
         <v>181</v>
@@ -1844,13 +1844,13 @@
         <v>182</v>
       </c>
       <c r="C3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D3" t="s">
         <v>182</v>
       </c>
       <c r="E3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F3" t="s">
         <v>182</v>
@@ -1865,13 +1865,13 @@
         <v>181</v>
       </c>
       <c r="J3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M3" t="s">
         <v>182</v>
@@ -1883,10 +1883,10 @@
         <v>181</v>
       </c>
       <c r="P3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R3" t="s">
         <v>181</v>
@@ -1901,7 +1901,7 @@
         <v>181</v>
       </c>
       <c r="V3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="W3" t="s">
         <v>181</v>
@@ -1913,25 +1913,25 @@
         <v>181</v>
       </c>
       <c r="Z3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AA3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AB3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AD3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AE3" t="s">
         <v>181</v>
       </c>
       <c r="AF3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AG3" t="s">
         <v>181</v>
@@ -1957,13 +1957,13 @@
         <v>181</v>
       </c>
       <c r="E4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H4" t="s">
         <v>182</v>
@@ -1981,25 +1981,25 @@
         <v>182</v>
       </c>
       <c r="M4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R4" t="s">
         <v>181</v>
       </c>
       <c r="S4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="T4" t="s">
         <v>181</v>
@@ -2011,13 +2011,13 @@
         <v>182</v>
       </c>
       <c r="W4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="X4" t="s">
         <v>181</v>
       </c>
       <c r="Y4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Z4" t="s">
         <v>181</v>
@@ -2026,7 +2026,7 @@
         <v>181</v>
       </c>
       <c r="AB4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC4" t="s">
         <v>181</v>
@@ -2035,16 +2035,16 @@
         <v>181</v>
       </c>
       <c r="AE4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AF4" t="s">
         <v>181</v>
       </c>
       <c r="AG4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AH4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AI4" t="s">
         <v>181</v>
@@ -2058,13 +2058,13 @@
         <v>182</v>
       </c>
       <c r="C5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F5" t="s">
         <v>181</v>
@@ -2073,10 +2073,10 @@
         <v>181</v>
       </c>
       <c r="H5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J5" t="s">
         <v>182</v>
@@ -2085,7 +2085,7 @@
         <v>181</v>
       </c>
       <c r="L5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M5" t="s">
         <v>182</v>
@@ -2097,19 +2097,19 @@
         <v>182</v>
       </c>
       <c r="P5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q5" t="s">
         <v>181</v>
       </c>
       <c r="R5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="T5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="U5" t="s">
         <v>182</v>
@@ -2118,7 +2118,7 @@
         <v>181</v>
       </c>
       <c r="W5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="X5" t="s">
         <v>181</v>
@@ -2127,13 +2127,13 @@
         <v>181</v>
       </c>
       <c r="Z5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AA5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AB5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC5" t="s">
         <v>181</v>
@@ -2142,19 +2142,19 @@
         <v>181</v>
       </c>
       <c r="AE5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AF5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AG5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AH5" t="s">
         <v>181</v>
       </c>
       <c r="AI5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6">
@@ -2165,31 +2165,31 @@
         <v>182</v>
       </c>
       <c r="C6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D6" t="s">
         <v>182</v>
       </c>
       <c r="E6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F6" t="s">
         <v>182</v>
       </c>
       <c r="G6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H6" t="s">
         <v>181</v>
       </c>
       <c r="I6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L6" t="s">
         <v>181</v>
@@ -2198,10 +2198,10 @@
         <v>181</v>
       </c>
       <c r="N6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P6" t="s">
         <v>182</v>
@@ -2210,7 +2210,7 @@
         <v>181</v>
       </c>
       <c r="R6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S6" t="s">
         <v>182</v>
@@ -2225,43 +2225,43 @@
         <v>181</v>
       </c>
       <c r="W6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="X6" t="s">
         <v>181</v>
       </c>
       <c r="Y6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Z6" t="s">
         <v>181</v>
       </c>
       <c r="AA6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AB6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AD6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AE6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AF6" t="s">
         <v>181</v>
       </c>
       <c r="AG6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AH6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AI6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7">
@@ -2272,10 +2272,10 @@
         <v>182</v>
       </c>
       <c r="C7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E7" t="s">
         <v>182</v>
@@ -2284,7 +2284,7 @@
         <v>181</v>
       </c>
       <c r="G7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H7" t="s">
         <v>182</v>
@@ -2302,43 +2302,43 @@
         <v>182</v>
       </c>
       <c r="M7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="T7" t="s">
         <v>182</v>
       </c>
       <c r="U7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="V7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="W7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="X7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Y7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Z7" t="s">
         <v>182</v>
@@ -2359,16 +2359,16 @@
         <v>181</v>
       </c>
       <c r="AF7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AG7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AH7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AI7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8">
@@ -2376,7 +2376,7 @@
         <v>188</v>
       </c>
       <c r="B8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C8" t="s">
         <v>182</v>
@@ -2385,22 +2385,22 @@
         <v>181</v>
       </c>
       <c r="E8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G8" t="s">
         <v>182</v>
       </c>
       <c r="H8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I8" t="s">
         <v>182</v>
       </c>
       <c r="J8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K8" t="s">
         <v>181</v>
@@ -2409,67 +2409,67 @@
         <v>181</v>
       </c>
       <c r="M8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N8" t="s">
         <v>181</v>
       </c>
       <c r="O8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q8" t="s">
         <v>182</v>
       </c>
       <c r="R8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="T8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="U8" t="s">
         <v>181</v>
       </c>
       <c r="V8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="W8" t="s">
         <v>182</v>
       </c>
       <c r="X8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Y8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Z8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AA8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AB8" t="s">
         <v>181</v>
       </c>
       <c r="AC8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AD8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AE8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AF8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AG8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AH8" t="s">
         <v>181</v>
@@ -2486,28 +2486,28 @@
         <v>182</v>
       </c>
       <c r="C9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D9" t="s">
         <v>182</v>
       </c>
       <c r="E9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H9" t="s">
         <v>182</v>
       </c>
       <c r="I9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K9" t="s">
         <v>182</v>
@@ -2516,7 +2516,7 @@
         <v>181</v>
       </c>
       <c r="M9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N9" t="s">
         <v>182</v>
@@ -2525,28 +2525,28 @@
         <v>181</v>
       </c>
       <c r="P9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q9" t="s">
         <v>181</v>
       </c>
       <c r="R9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="T9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="U9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="V9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="W9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="X9" t="s">
         <v>182</v>
@@ -2555,31 +2555,31 @@
         <v>181</v>
       </c>
       <c r="Z9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AA9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AB9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC9" t="s">
         <v>181</v>
       </c>
       <c r="AD9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AE9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AF9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AG9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AH9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AI9" t="s">
         <v>181</v>

</xml_diff>